<commit_message>
feat(employee): update PF calculation formulas and text names to match PF.xlsx template
</commit_message>
<xml_diff>
--- a/web/templates/PF.xlsx
+++ b/web/templates/PF.xlsx
@@ -1,18 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9303"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ujjawal\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A36003-E379-4AFC-A840-BCA35AEF4A2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="19425" windowHeight="10305" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{C4D77260-AA67-4067-AC4A-E3C888662E79}"/>
   </bookViews>
   <sheets>
-    <sheet name="YES" sheetId="1" r:id="rId1"/>
-    <sheet name="NO" sheetId="2" r:id="rId2"/>
+    <sheet name="PF Applied" sheetId="1" r:id="rId1"/>
+    <sheet name="Out out from PF" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">NO!$B$2:$D$17</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">YES!$B$2:$D$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Out out from PF'!$B$2:$D$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'PF Applied'!$B$2:$D$17</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -86,7 +92,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
@@ -356,10 +362,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -669,25 +675,25 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:G17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4008F73A-4EF5-401F-9FC3-10DEA3A02279}">
+  <dimension ref="B2:I17"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
         <v>4</v>
       </c>
@@ -697,19 +703,23 @@
         <v>5</v>
       </c>
       <c r="G2" s="2">
-        <v>512000</v>
-      </c>
-    </row>
-    <row r="3" spans="2:7" thickBot="1" x14ac:dyDescent="0.4">
+        <v>504000</v>
+      </c>
+      <c r="I2">
+        <f>42000*12</f>
+        <v>504000</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F3" t="s">
         <v>6</v>
       </c>
       <c r="G3" s="3">
         <f>G2/12</f>
-        <v>42666.666666666664</v>
-      </c>
-    </row>
-    <row r="4" spans="2:7" thickBot="1" x14ac:dyDescent="0.4">
+        <v>42000</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="11" t="s">
         <v>14</v>
       </c>
@@ -720,136 +730,136 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
       <c r="C5" s="14">
-        <f>IF(G3&lt;42000,MIN(21500,G3),G3/2)</f>
-        <v>21333.333333333332</v>
+        <f>IF(G3&lt;=42000,MIN(21500,G3),G3/2)</f>
+        <v>21500</v>
       </c>
       <c r="D5" s="5">
         <f>C5*12</f>
-        <v>256000</v>
-      </c>
-    </row>
-    <row r="6" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+        <v>258000</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C6" s="14">
         <f>IF(G3&lt;42000,G3-C5-C8,C5/2)</f>
-        <v>10666.666666666666</v>
+        <v>10750</v>
       </c>
       <c r="D6" s="5">
         <f t="shared" ref="D6:D9" si="0">C6*12</f>
-        <v>128000</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+        <v>129000</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>2</v>
       </c>
       <c r="C7" s="14">
         <f>ROUND(IF(G3&lt;42000,0,G3*10%),0)</f>
-        <v>4267</v>
+        <v>4200</v>
       </c>
       <c r="D7" s="5">
         <f t="shared" si="0"/>
-        <v>51204</v>
-      </c>
-    </row>
-    <row r="8" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+        <v>50400</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="14">
-        <f>ROUND(IF(C5&gt;15000,1800,C5*12%),0)</f>
-        <v>1800</v>
+        <f>ROUND(IF(C5&gt;25000,3000,C5*12%),0)</f>
+        <v>2580</v>
       </c>
       <c r="D8" s="5">
         <f t="shared" si="0"/>
-        <v>21600</v>
-      </c>
-    </row>
-    <row r="9" spans="2:7" thickBot="1" x14ac:dyDescent="0.4">
+        <v>30960</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C9" s="15">
         <f>(G3-SUM(C5:C8))</f>
-        <v>4599.6666666666642</v>
+        <v>2970</v>
       </c>
       <c r="D9" s="9">
         <f t="shared" si="0"/>
-        <v>55195.999999999971</v>
-      </c>
-    </row>
-    <row r="10" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+        <v>35640</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C10" s="14">
         <f>SUM(C5:C9)</f>
-        <v>42666.666666666664</v>
+        <v>42000</v>
       </c>
       <c r="D10" s="5">
         <f>SUM(D5:D9)</f>
-        <v>512000</v>
-      </c>
-    </row>
-    <row r="11" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+        <v>504000</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="10" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="6"/>
     </row>
-    <row r="12" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C12" s="17">
         <f>C8</f>
-        <v>1800</v>
+        <v>2580</v>
       </c>
       <c r="D12" s="5">
         <f t="shared" ref="D12:D13" si="1">C12*12</f>
-        <v>21600</v>
-      </c>
-    </row>
-    <row r="13" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+        <v>30960</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C13" s="22">
         <f>C12</f>
-        <v>1800</v>
+        <v>2580</v>
       </c>
       <c r="D13" s="23">
         <f t="shared" si="1"/>
-        <v>21600</v>
-      </c>
-    </row>
-    <row r="14" spans="2:7" thickBot="1" x14ac:dyDescent="0.4">
+        <v>30960</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="19" t="s">
         <v>13</v>
       </c>
       <c r="C14" s="20">
         <f>C10-SUM(C12:C13)</f>
-        <v>39066.666666666664</v>
+        <v>36840</v>
       </c>
       <c r="D14" s="21">
         <f>D10-SUM(D12:D13)</f>
-        <v>468800</v>
-      </c>
-    </row>
-    <row r="15" spans="2:7" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+        <v>442080</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="7"/>
       <c r="C15" s="18"/>
       <c r="D15" s="8"/>
     </row>
-    <row r="16" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="25" t="s">
         <v>15</v>
       </c>
@@ -872,18 +882,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78AD73DD-FF83-4B5D-9C41-2D8B2F74F4A5}">
   <dimension ref="B2:G17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.28515625" customWidth="1"/>
     <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
         <v>4</v>
       </c>
@@ -896,7 +906,7 @@
         <v>276000</v>
       </c>
     </row>
-    <row r="3" spans="2:7" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F3" t="s">
         <v>6</v>
       </c>
@@ -905,7 +915,7 @@
         <v>23000</v>
       </c>
     </row>
-    <row r="4" spans="2:7" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="11" t="s">
         <v>14</v>
       </c>
@@ -916,7 +926,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
@@ -929,7 +939,7 @@
         <v>258000</v>
       </c>
     </row>
-    <row r="6" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>1</v>
       </c>
@@ -942,7 +952,7 @@
         <v>18000</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>2</v>
       </c>
@@ -955,7 +965,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
         <v>7</v>
       </c>
@@ -967,7 +977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:7" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="7" t="s">
         <v>3</v>
       </c>
@@ -980,7 +990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="4" t="s">
         <v>10</v>
       </c>
@@ -993,14 +1003,14 @@
         <v>276000</v>
       </c>
     </row>
-    <row r="11" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" s="10" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="6"/>
     </row>
-    <row r="12" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="4" t="s">
         <v>7</v>
       </c>
@@ -1013,7 +1023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:7" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="4" t="s">
         <v>12</v>
       </c>
@@ -1026,7 +1036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:7" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="19" t="s">
         <v>13</v>
       </c>
@@ -1039,7 +1049,7 @@
         <v>276000</v>
       </c>
     </row>
-    <row r="15" spans="2:7" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="7"/>
       <c r="C15" s="18"/>
       <c r="D15" s="8"/>

</xml_diff>